<commit_message>
Add new project page for personal portfolio and include FileSorter presentation PDF
</commit_message>
<xml_diff>
--- a/assets/docs/E5_Tableau-de-synthese.xlsx
+++ b/assets/docs/E5_Tableau-de-synthese.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/63129c17ad4e6253/Desktop/Portfolio/assets/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samur\OneDrive\Desktop\Portfolio\assets\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="8_{54BF382C-933A-4DD1-91D6-261A13667A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90786083-CEA6-4FD7-8927-E71F11681785}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2299F28B-55EB-4CAF-B7D0-DC9FF05A4BFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$30</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="39">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -132,9 +132,6 @@
     <t>Réalisations en milieu professionnel en cours de seconde année</t>
   </si>
   <si>
-    <t>03/09/2025 au 14/04/2026</t>
-  </si>
-  <si>
     <t>NOM et prénom : Boutin Samuel</t>
   </si>
   <si>
@@ -144,56 +141,40 @@
     <t>Adresse URL du portfolio : portfolio.rustevolution.net</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Conception et déploiement d'une solution numérique pour supprimer le suivi papier des astreintes du pôle CFA, création d'interfaces de saisie structurées, développement d'un rapport d'intervention automatisé via Crystal Reports et mise en place d'un workflow d'envoi automatique par email à la clôture des bons d'intervention,
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Documents / productions associées:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Écran de saisie personnalisé ASTREINTE_CFA
-Configuration du Plugin Mail
-Rapport automatique SAP Crystal Report (PAH_CFA_Astreinte_V2)
-Documentation utilisateur (Guide de prise en main)</t>
-    </r>
-  </si>
-  <si>
-    <t>Du 01/11/2025 au 09/03/2026</t>
-  </si>
-  <si>
     <t>x</t>
   </si>
   <si>
     <t>Portfolio</t>
   </si>
   <si>
-    <t>01/01/2017 au 01/07/2024</t>
-  </si>
-  <si>
     <t>Site E-Commerce Wordpress</t>
   </si>
   <si>
-    <t>Projet Minecraft JAVA</t>
-  </si>
-  <si>
-    <t>Site de recrutement FIVEM</t>
-  </si>
-  <si>
-    <t>Leaderboard</t>
+    <t>NAS Synology sécurisé avec OpenVPN</t>
+  </si>
+  <si>
+    <t>01/11/2025 au 09/03/2026</t>
+  </si>
+  <si>
+    <t>26/05/2026 à aujourd'hui</t>
+  </si>
+  <si>
+    <t>Coswin 8i12 – Paramétrage et digitalisation du suivi des astreintes CFA</t>
+  </si>
+  <si>
+    <t>Jaspersoft Studio – Conception et déploiement d’un rapport de suivi des astreintes CFA</t>
+  </si>
+  <si>
+    <t>CFA – Publication du rapport sur Jaspersoft Server</t>
+  </si>
+  <si>
+    <t>20/07/2026 à aujourd'hui</t>
+  </si>
+  <si>
+    <t>01/01/2017 à aujourd'hui</t>
+  </si>
+  <si>
+    <t>03/09/2025 à aujourd'hui</t>
   </si>
 </sst>
 </file>
@@ -203,7 +184,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -266,13 +247,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <u/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="72"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -286,7 +260,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="31">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -670,6 +644,19 @@
       <bottom style="medium">
         <color theme="2" tint="-0.749992370372631"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </left>
+      <right style="medium">
+        <color theme="2" tint="-0.749992370372631"/>
+      </right>
+      <top style="medium">
+        <color theme="2" tint="-0.749992370372631"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -683,20 +670,22 @@
         <color indexed="64"/>
       </top>
       <bottom style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
       </left>
       <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
+        <color indexed="64"/>
       </right>
-      <top/>
+      <top style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </top>
       <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -778,19 +767,22 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -808,7 +800,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -861,9 +853,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -888,15 +877,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>256860</xdr:colOff>
+      <xdr:colOff>603224</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>141555</xdr:rowOff>
+      <xdr:rowOff>127701</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>371995</xdr:colOff>
+      <xdr:colOff>718359</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>301755</xdr:rowOff>
+      <xdr:rowOff>287901</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
       <mc:Choice Requires="xdr14">
@@ -913,8 +902,8 @@
           </xdr14:nvContentPartPr>
           <xdr14:nvPr macro=""/>
           <xdr14:xfrm>
-            <a:off x="13401360" y="1675080"/>
-            <a:ext cx="111960" cy="160200"/>
+            <a:off x="16425115" y="1637846"/>
+            <a:ext cx="115135" cy="160200"/>
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
@@ -1288,7 +1277,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ81"/>
+  <dimension ref="A1:AQ76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.77734375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="72.6640625" style="1" customWidth="1"/>
@@ -1303,56 +1292,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30" t="s">
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="30"/>
+      <c r="H1" s="31"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
     </row>
     <row r="3" spans="1:43" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="43" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" s="44"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="49" t="s">
+      <c r="A3" s="44" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="44"/>
-      <c r="H3" s="50"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="51"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="46" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="47"/>
-      <c r="C4" s="47"/>
-      <c r="D4" s="47"/>
-      <c r="E4" s="48"/>
+      <c r="A4" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="49"/>
       <c r="F4" s="12" t="s">
         <v>4</v>
       </c>
@@ -1364,22 +1353,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="41"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="42"/>
+      <c r="A5" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="43"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="39" t="s">
         <v>8</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1402,8 +1391,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="325.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="29"/>
-      <c r="B7" s="39"/>
+      <c r="A7" s="30"/>
+      <c r="B7" s="40"/>
       <c r="C7" s="18" t="s">
         <v>15</v>
       </c>
@@ -1459,16 +1448,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="32"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="33"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="34"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1506,27 +1495,25 @@
       <c r="AQ8"/>
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A9" s="51" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="27" t="s">
-        <v>30</v>
-      </c>
+      <c r="A9" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="24"/>
       <c r="D9" s="21"/>
-      <c r="E9" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="F9" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="G9" s="27" t="s">
-        <v>30</v>
+      <c r="E9" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="26" t="s">
+        <v>27</v>
       </c>
       <c r="H9" s="27" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="I9"/>
       <c r="J9"/>
@@ -1565,30 +1552,28 @@
       <c r="AQ9"/>
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A10" s="51" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="E10" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="F10" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="G10" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="H10" s="27" t="s">
-        <v>30</v>
-      </c>
+      <c r="A10" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="28"/>
       <c r="I10"/>
       <c r="J10"/>
       <c r="K10"/>
@@ -1626,24 +1611,24 @@
       <c r="AQ10"/>
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A11" s="51" t="s">
-        <v>34</v>
-      </c>
-      <c r="B11" s="8"/>
-      <c r="C11" s="27" t="s">
+      <c r="A11" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="21"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>27</v>
+      </c>
       <c r="E11" s="21"/>
-      <c r="F11" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="G11" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="H11" s="27" t="s">
-        <v>30</v>
-      </c>
+      <c r="F11" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" s="22"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1680,27 +1665,15 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A12" s="51" t="s">
-        <v>35</v>
-      </c>
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="25"/>
       <c r="B12" s="8"/>
       <c r="C12" s="21"/>
-      <c r="D12" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="F12" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="G12" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="H12" s="27" t="s">
-        <v>30</v>
-      </c>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="22"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1737,24 +1710,14 @@
       <c r="AP12"/>
       <c r="AQ12"/>
     </row>
-    <row r="13" spans="1:43" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A13" s="51" t="s">
-        <v>36</v>
-      </c>
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="25"/>
       <c r="B13" s="8"/>
-      <c r="C13" s="27" t="s">
-        <v>30</v>
-      </c>
+      <c r="C13" s="21"/>
       <c r="D13" s="21"/>
-      <c r="E13" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="F13" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="G13" s="27" t="s">
-        <v>30</v>
-      </c>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
       <c r="H13" s="22"/>
       <c r="I13"/>
       <c r="J13"/>
@@ -1792,15 +1755,17 @@
       <c r="AP13"/>
       <c r="AQ13"/>
     </row>
-    <row r="14" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="51"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="22"/>
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A14" s="35" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="36"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="37"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="38"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1837,15 +1802,25 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="51"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="22"/>
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="A15" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="G15" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="H15" s="15"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1882,15 +1857,25 @@
       <c r="AP15"/>
       <c r="AQ15"/>
     </row>
-    <row r="16" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="51"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="22"/>
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="A16" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="14"/>
+      <c r="D16" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" s="14"/>
+      <c r="F16" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="G16" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="H16" s="15"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1927,15 +1912,25 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="51"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="22"/>
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="A17" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="14"/>
+      <c r="D17" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" s="14"/>
+      <c r="F17" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="G17" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="H17" s="15"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1973,14 +1968,14 @@
       <c r="AQ17"/>
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="51"/>
+      <c r="A18" s="25"/>
       <c r="B18" s="8"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="22"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="15"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -2017,17 +2012,15 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A19" s="34" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="35"/>
-      <c r="C19" s="36"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="36"/>
-      <c r="F19" s="36"/>
-      <c r="G19" s="36"/>
-      <c r="H19" s="37"/>
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="25"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="15"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -2064,29 +2057,15 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="145.80000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="B20" s="26" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="D20" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="G20" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="H20" s="27" t="s">
-        <v>30</v>
-      </c>
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="25"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="15"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -2124,8 +2103,8 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="9"/>
-      <c r="B21" s="25"/>
+      <c r="A21" s="25"/>
+      <c r="B21" s="8"/>
       <c r="C21" s="14"/>
       <c r="D21" s="14"/>
       <c r="E21" s="14"/>
@@ -2168,15 +2147,17 @@
       <c r="AP21"/>
       <c r="AQ21"/>
     </row>
-    <row r="22" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="9"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="15"/>
+    <row r="22" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A22" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="37"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="38"/>
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -2393,17 +2374,15 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A27" s="34" t="s">
-        <v>23</v>
-      </c>
-      <c r="B27" s="36"/>
-      <c r="C27" s="36"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="36"/>
-      <c r="F27" s="36"/>
-      <c r="G27" s="36"/>
-      <c r="H27" s="37"/>
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="9"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="15"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2485,15 +2464,15 @@
       <c r="AP28"/>
       <c r="AQ28"/>
     </row>
-    <row r="29" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="9"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="15"/>
+    <row r="29" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="10"/>
+      <c r="B29" s="11"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="17"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2530,15 +2509,15 @@
       <c r="AP29"/>
       <c r="AQ29"/>
     </row>
-    <row r="30" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="9"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="15"/>
+    <row r="30" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A30" s="5"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2575,244 +2554,24 @@
       <c r="AP30"/>
       <c r="AQ30"/>
     </row>
-    <row r="31" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="9"/>
-      <c r="B31" s="8"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="15"/>
-      <c r="I31"/>
-      <c r="J31"/>
-      <c r="K31"/>
-      <c r="L31"/>
-      <c r="M31"/>
-      <c r="N31"/>
-      <c r="O31"/>
-      <c r="P31"/>
-      <c r="Q31"/>
-      <c r="R31"/>
-      <c r="S31"/>
-      <c r="T31"/>
-      <c r="U31"/>
-      <c r="V31"/>
-      <c r="W31"/>
-      <c r="X31"/>
-      <c r="Y31"/>
-      <c r="Z31"/>
-      <c r="AA31"/>
-      <c r="AB31"/>
-      <c r="AC31"/>
-      <c r="AD31"/>
-      <c r="AE31"/>
-      <c r="AF31"/>
-      <c r="AG31"/>
-      <c r="AH31"/>
-      <c r="AI31"/>
-      <c r="AJ31"/>
-      <c r="AK31"/>
-      <c r="AL31"/>
-      <c r="AM31"/>
-      <c r="AN31"/>
-      <c r="AO31"/>
-      <c r="AP31"/>
-      <c r="AQ31"/>
-    </row>
-    <row r="32" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="9"/>
-      <c r="B32" s="8"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="15"/>
-      <c r="I32"/>
-      <c r="J32"/>
-      <c r="K32"/>
-      <c r="L32"/>
-      <c r="M32"/>
-      <c r="N32"/>
-      <c r="O32"/>
-      <c r="P32"/>
-      <c r="Q32"/>
-      <c r="R32"/>
-      <c r="S32"/>
-      <c r="T32"/>
-      <c r="U32"/>
-      <c r="V32"/>
-      <c r="W32"/>
-      <c r="X32"/>
-      <c r="Y32"/>
-      <c r="Z32"/>
-      <c r="AA32"/>
-      <c r="AB32"/>
-      <c r="AC32"/>
-      <c r="AD32"/>
-      <c r="AE32"/>
-      <c r="AF32"/>
-      <c r="AG32"/>
-      <c r="AH32"/>
-      <c r="AI32"/>
-      <c r="AJ32"/>
-      <c r="AK32"/>
-      <c r="AL32"/>
-      <c r="AM32"/>
-      <c r="AN32"/>
-      <c r="AO32"/>
-      <c r="AP32"/>
-      <c r="AQ32"/>
-    </row>
-    <row r="33" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="9"/>
-      <c r="B33" s="8"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="15"/>
-      <c r="I33"/>
-      <c r="J33"/>
-      <c r="K33"/>
-      <c r="L33"/>
-      <c r="M33"/>
-      <c r="N33"/>
-      <c r="O33"/>
-      <c r="P33"/>
-      <c r="Q33"/>
-      <c r="R33"/>
-      <c r="S33"/>
-      <c r="T33"/>
-      <c r="U33"/>
-      <c r="V33"/>
-      <c r="W33"/>
-      <c r="X33"/>
-      <c r="Y33"/>
-      <c r="Z33"/>
-      <c r="AA33"/>
-      <c r="AB33"/>
-      <c r="AC33"/>
-      <c r="AD33"/>
-      <c r="AE33"/>
-      <c r="AF33"/>
-      <c r="AG33"/>
-      <c r="AH33"/>
-      <c r="AI33"/>
-      <c r="AJ33"/>
-      <c r="AK33"/>
-      <c r="AL33"/>
-      <c r="AM33"/>
-      <c r="AN33"/>
-      <c r="AO33"/>
-      <c r="AP33"/>
-      <c r="AQ33"/>
-    </row>
-    <row r="34" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="10"/>
-      <c r="B34" s="11"/>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="16"/>
-      <c r="H34" s="17"/>
-      <c r="I34"/>
-      <c r="J34"/>
-      <c r="K34"/>
-      <c r="L34"/>
-      <c r="M34"/>
-      <c r="N34"/>
-      <c r="O34"/>
-      <c r="P34"/>
-      <c r="Q34"/>
-      <c r="R34"/>
-      <c r="S34"/>
-      <c r="T34"/>
-      <c r="U34"/>
-      <c r="V34"/>
-      <c r="W34"/>
-      <c r="X34"/>
-      <c r="Y34"/>
-      <c r="Z34"/>
-      <c r="AA34"/>
-      <c r="AB34"/>
-      <c r="AC34"/>
-      <c r="AD34"/>
-      <c r="AE34"/>
-      <c r="AF34"/>
-      <c r="AG34"/>
-      <c r="AH34"/>
-      <c r="AI34"/>
-      <c r="AJ34"/>
-      <c r="AK34"/>
-      <c r="AL34"/>
-      <c r="AM34"/>
-      <c r="AN34"/>
-      <c r="AO34"/>
-      <c r="AP34"/>
-      <c r="AQ34"/>
-    </row>
-    <row r="35" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A35" s="5"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35"/>
-      <c r="J35"/>
-      <c r="K35"/>
-      <c r="L35"/>
-      <c r="M35"/>
-      <c r="N35"/>
-      <c r="O35"/>
-      <c r="P35"/>
-      <c r="Q35"/>
-      <c r="R35"/>
-      <c r="S35"/>
-      <c r="T35"/>
-      <c r="U35"/>
-      <c r="V35"/>
-      <c r="W35"/>
-      <c r="X35"/>
-      <c r="Y35"/>
-      <c r="Z35"/>
-      <c r="AA35"/>
-      <c r="AB35"/>
-      <c r="AC35"/>
-      <c r="AD35"/>
-      <c r="AE35"/>
-      <c r="AF35"/>
-      <c r="AG35"/>
-      <c r="AH35"/>
-      <c r="AI35"/>
-      <c r="AJ35"/>
-      <c r="AK35"/>
-      <c r="AL35"/>
-      <c r="AM35"/>
-      <c r="AN35"/>
-      <c r="AO35"/>
-      <c r="AP35"/>
-      <c r="AQ35"/>
-    </row>
-    <row r="36" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="33" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="34" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="35" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="36" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="37" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="38" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="39" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="40" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="41" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="42" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="44" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="45" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="46" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="47" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="48" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="49" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="50" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="51" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -2841,11 +2600,6 @@
     <row r="74" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="75" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="76" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="77" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="78" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="79" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="80" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="G1:H1"/>
@@ -2856,8 +2610,8 @@
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A22:H22"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
   </mergeCells>

</xml_diff>

<commit_message>
Update E5_Tableau-de-synthese.xlsx with new data
</commit_message>
<xml_diff>
--- a/assets/docs/E5_Tableau-de-synthese.xlsx
+++ b/assets/docs/E5_Tableau-de-synthese.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samur\OneDrive\Desktop\Portfolio\assets\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2299F28B-55EB-4CAF-B7D0-DC9FF05A4BFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2755640F-2C93-4DB2-A5CF-FF57F289EB85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="39">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -785,15 +785,39 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -828,30 +852,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1292,56 +1292,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31" t="s">
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="31"/>
+      <c r="H1" s="29"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
     </row>
     <row r="3" spans="1:43" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="44" t="s">
+      <c r="A3" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="50" t="s">
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="45"/>
-      <c r="H3" s="51"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="37"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="49"/>
+      <c r="B4" s="34"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="35"/>
       <c r="F4" s="12" t="s">
         <v>4</v>
       </c>
@@ -1353,22 +1353,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="49" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
+      <c r="B5" s="50"/>
+      <c r="C5" s="50"/>
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="50"/>
+      <c r="G5" s="50"/>
+      <c r="H5" s="51"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="47" t="s">
         <v>8</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1391,8 +1391,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="325.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="30"/>
-      <c r="B7" s="40"/>
+      <c r="A7" s="39"/>
+      <c r="B7" s="48"/>
       <c r="C7" s="18" t="s">
         <v>15</v>
       </c>
@@ -1448,16 +1448,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="34"/>
+      <c r="B8" s="41"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="41"/>
+      <c r="F8" s="41"/>
+      <c r="G8" s="41"/>
+      <c r="H8" s="42"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1618,9 +1618,7 @@
       <c r="C11" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="24" t="s">
-        <v>27</v>
-      </c>
+      <c r="D11" s="24"/>
       <c r="E11" s="21"/>
       <c r="F11" s="24" t="s">
         <v>27</v>
@@ -1756,16 +1754,16 @@
       <c r="AQ13"/>
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A14" s="35" t="s">
+      <c r="A14" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="36"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="37"/>
-      <c r="G14" s="37"/>
-      <c r="H14" s="38"/>
+      <c r="B14" s="44"/>
+      <c r="C14" s="45"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="45"/>
+      <c r="G14" s="45"/>
+      <c r="H14" s="46"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -2148,16 +2146,16 @@
       <c r="AQ21"/>
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A22" s="35" t="s">
+      <c r="A22" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="37"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="37"/>
-      <c r="F22" s="37"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="38"/>
+      <c r="B22" s="45"/>
+      <c r="C22" s="45"/>
+      <c r="D22" s="45"/>
+      <c r="E22" s="45"/>
+      <c r="F22" s="45"/>
+      <c r="G22" s="45"/>
+      <c r="H22" s="46"/>
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -2602,11 +2600,6 @@
     <row r="76" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2614,6 +2607,11 @@
     <mergeCell ref="A22:H22"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2634,6 +2632,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="78f9c018-01b4-440e-aee1-76a45e3ac1b8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="08be48cc-634c-4395-a031-931afa9b2f2b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002324AC850D2DCA4DAEA93F87C0CCAB13" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="53945bb04d5e8a952e817e21b06ad93d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="78f9c018-01b4-440e-aee1-76a45e3ac1b8" xmlns:ns3="08be48cc-634c-4395-a031-931afa9b2f2b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c4f49df68ea2ccf9041bd7533fbae066" ns2:_="" ns3:_="">
     <xsd:import namespace="78f9c018-01b4-440e-aee1-76a45e3ac1b8"/>
@@ -2822,17 +2831,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="78f9c018-01b4-440e-aee1-76a45e3ac1b8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="08be48cc-634c-4395-a031-931afa9b2f2b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A0F5447-1756-4C3A-A844-A0D3A2CADE36}">
   <ds:schemaRefs>
@@ -2842,6 +2840,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1B0686C-7B7C-4AA8-9920-42B46C3627A2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="78f9c018-01b4-440e-aee1-76a45e3ac1b8"/>
+    <ds:schemaRef ds:uri="08be48cc-634c-4395-a031-931afa9b2f2b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95B9F24E-D13B-48CE-9198-01F130491792}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2858,15 +2867,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1B0686C-7B7C-4AA8-9920-42B46C3627A2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="78f9c018-01b4-440e-aee1-76a45e3ac1b8"/>
-    <ds:schemaRef ds:uri="08be48cc-634c-4395-a031-931afa9b2f2b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update CV_Samuel_Boutin.pdf and E5_Tableau-de-synthese.xlsx with new information
</commit_message>
<xml_diff>
--- a/assets/docs/E5_Tableau-de-synthese.xlsx
+++ b/assets/docs/E5_Tableau-de-synthese.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samur\OneDrive\Desktop\Portfolio\assets\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samur\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2755640F-2C93-4DB2-A5CF-FF57F289EB85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25ECD5D0-2C31-4B97-92E4-F53826192BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,12 +39,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="42">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
-  </si>
-  <si>
-    <t>SESSION 2026</t>
   </si>
   <si>
     <t xml:space="preserve">Tableau de synthèse des réalisations professionnelles </t>
@@ -175,6 +172,18 @@
   </si>
   <si>
     <t>03/09/2025 à aujourd'hui</t>
+  </si>
+  <si>
+    <t>04/06/2026 au 10/06/2026</t>
+  </si>
+  <si>
+    <t>Conception et déploiement d'un outil Python de classement intelligent des ressources pédagogiques avec Ollama.</t>
+  </si>
+  <si>
+    <t>20/04/2026 au 23/04/2026</t>
+  </si>
+  <si>
+    <t>SESSION 2025-2027</t>
   </si>
 </sst>
 </file>
@@ -785,9 +794,51 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -810,48 +861,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1292,124 +1301,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29" t="s">
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="31"/>
+    </row>
+    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="29"/>
-    </row>
-    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+    </row>
+    <row r="3" spans="1:43" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="44" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-    </row>
-    <row r="3" spans="1:43" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="30" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="36" t="s">
-        <v>3</v>
-      </c>
-      <c r="G3" s="31"/>
-      <c r="H3" s="37"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="51"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="49"/>
+      <c r="F4" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4" s="20" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:43" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="G4" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" s="20" t="s">
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="43"/>
+    </row>
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="29" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:43" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="49" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="50"/>
-      <c r="C5" s="50"/>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="50"/>
-      <c r="H5" s="51"/>
-    </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="38" t="s">
+      <c r="B6" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="47" t="s">
+      <c r="C6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="7" t="s">
+    </row>
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="325.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="30"/>
+      <c r="B7" s="40"/>
+      <c r="C7" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="325.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="39"/>
-      <c r="B7" s="48"/>
-      <c r="C7" s="18" t="s">
+      <c r="D7" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="E7" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="F7" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="G7" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="H7" s="19" t="s">
         <v>19</v>
-      </c>
-      <c r="H7" s="19" t="s">
-        <v>20</v>
       </c>
       <c r="I7"/>
       <c r="J7"/>
@@ -1448,16 +1457,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="41"/>
-      <c r="C8" s="41"/>
-      <c r="D8" s="41"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="41"/>
-      <c r="G8" s="41"/>
-      <c r="H8" s="42"/>
+      <c r="A8" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="34"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1496,24 +1505,24 @@
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C9" s="24"/>
       <c r="D9" s="21"/>
       <c r="E9" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G9" s="26" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H9" s="27" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I9"/>
       <c r="J9"/>
@@ -1553,25 +1562,25 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G10" s="26" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H10" s="28"/>
       <c r="I10"/>
@@ -1612,19 +1621,21 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" s="23"/>
+        <v>29</v>
+      </c>
+      <c r="B11" s="23" t="s">
+        <v>38</v>
+      </c>
       <c r="C11" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D11" s="24"/>
       <c r="E11" s="21"/>
       <c r="F11" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H11" s="22"/>
       <c r="I11"/>
@@ -1663,15 +1674,25 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="25"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="21"/>
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+      <c r="A12" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>26</v>
+      </c>
       <c r="D12" s="21"/>
       <c r="E12" s="21"/>
       <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
-      <c r="H12" s="22"/>
+      <c r="G12" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="H12" s="24" t="s">
+        <v>26</v>
+      </c>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1754,16 +1775,16 @@
       <c r="AQ13"/>
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A14" s="43" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" s="44"/>
-      <c r="C14" s="45"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="46"/>
+      <c r="A14" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="36"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="37"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="38"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1802,21 +1823,21 @@
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A15" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C15" s="24"/>
       <c r="D15" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E15" s="24"/>
       <c r="F15" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H15" s="15"/>
       <c r="I15"/>
@@ -1857,21 +1878,21 @@
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A16" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E16" s="14"/>
       <c r="F16" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H16" s="15"/>
       <c r="I16"/>
@@ -1912,21 +1933,21 @@
     </row>
     <row r="17" spans="1:43" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="A17" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="23" t="s">
         <v>35</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>36</v>
       </c>
       <c r="C17" s="14"/>
       <c r="D17" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E17" s="14"/>
       <c r="F17" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G17" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H17" s="15"/>
       <c r="I17"/>
@@ -2146,16 +2167,16 @@
       <c r="AQ21"/>
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A22" s="43" t="s">
-        <v>23</v>
-      </c>
-      <c r="B22" s="45"/>
-      <c r="C22" s="45"/>
-      <c r="D22" s="45"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45"/>
-      <c r="H22" s="46"/>
+      <c r="A22" s="35" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="37"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="38"/>
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -2600,6 +2621,11 @@
     <row r="76" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2607,11 +2633,6 @@
     <mergeCell ref="A22:H22"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2623,15 +2644,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="78f9c018-01b4-440e-aee1-76a45e3ac1b8">
@@ -2640,6 +2652,15 @@
     <TaxCatchAll xmlns="08be48cc-634c-4395-a031-931afa9b2f2b" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2832,20 +2853,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A0F5447-1756-4C3A-A844-A0D3A2CADE36}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1B0686C-7B7C-4AA8-9920-42B46C3627A2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="78f9c018-01b4-440e-aee1-76a45e3ac1b8"/>
     <ds:schemaRef ds:uri="08be48cc-634c-4395-a031-931afa9b2f2b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A0F5447-1756-4C3A-A844-A0D3A2CADE36}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>